<commit_message>
hardware: 3D-printable enclosure + JLCPCB fab fixes
- case/: parametric OpenSCAD clamshell (lumigate_case.scad) driven by the live
  PCB (extract_case_params.py) + measured connector heights; XLR flange screw
  holes corrected to the datasheet diagonal pattern (M2, 12.5mm centre); STL +
  assembly GLB deliverables, Blender doc renders.
- gen_gerbers.py: board-safe fab export (kicad-cli, ALWAYS aux/drill origin) so
  gerbers + CPL share the bottom-left origin (fixes JLCPCB "parts off the board").
- BOM: J4 = C160408 (JST SM09B-SRSS-TB, in stock); group by LCSC# (one line per
  part); fee-free swaps D4 yellow -> C89811 (preferred), R18 49.9R -> C25120 (basic).
- gerbers re-exported with aux origin; CPL .xlsx regenerated with J4.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/lumigate_CPL.xlsx
+++ b/hardware/lumigate_CPL.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,12 +451,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>13.2389mm</t>
+          <t>15.1690mm</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10.5750mm</t>
+          <t>9.0828mm</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>14.0750mm</t>
+          <t>12.5750mm</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>12.5750mm</t>
+          <t>11.0750mm</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>42.2389mm</t>
+          <t>43.2389mm</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>16.5750mm</t>
+          <t>16.0750mm</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -551,12 +551,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>45.2389mm</t>
+          <t>45.7389mm</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>16.5750mm</t>
+          <t>18.5750mm</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -576,12 +576,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>48.2389mm</t>
+          <t>50.7389mm</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>22.5750mm</t>
+          <t>24.0750mm</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11.0750mm</t>
+          <t>9.0750mm</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>5.0750mm</t>
+          <t>3.5750mm</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>5.0750mm</t>
+          <t>3.5750mm</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>47.7189mm</t>
+          <t>48.7189mm</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5.0750mm</t>
+          <t>3.5750mm</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>51.2189mm</t>
+          <t>52.2189mm</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -776,12 +776,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>31.2189mm</t>
+          <t>28.7189mm</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7.1000mm</t>
+          <t>6.6000mm</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -851,12 +851,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>39.7389mm</t>
+          <t>42.2389mm</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10.5750mm</t>
+          <t>11.0750mm</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>17.0750mm</t>
+          <t>16.5750mm</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>15.5750mm</t>
+          <t>14.5750mm</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -976,12 +976,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>51.2189mm</t>
+          <t>51.7689mm</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>37.6375mm</t>
+          <t>38.0125mm</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>39.8889mm</t>
+          <t>37.5489mm</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1196,17 +1196,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>23.1189mm</t>
+          <t>29.2189mm</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16.0750mm</t>
+          <t>30.5750mm</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1215,23 +1215,23 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PS1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>39.1989mm</t>
+          <t>24.1189mm</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>43.9950mm</t>
+          <t>22.0750mm</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1246,17 +1246,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>PS1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>9.6564mm</t>
+          <t>41.6989mm</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>13.6250mm</t>
+          <t>44.4950mm</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1265,13 +1265,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17.6250mm</t>
+          <t>13.6250mm</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1296,17 +1296,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>13.2089mm</t>
+          <t>9.6564mm</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>16.5750mm</t>
+          <t>17.6250mm</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1315,23 +1315,23 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>38.2089mm</t>
+          <t>15.1590mm</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23.5750mm</t>
+          <t>15.0828mm</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1346,12 +1346,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>31.7089mm</t>
+          <t>38.2089mm</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1365,23 +1365,23 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>51.6314mm</t>
+          <t>31.7089mm</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>33.0750mm</t>
+          <t>23.5750mm</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1396,17 +1396,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2.7189mm</t>
+          <t>51.6314mm</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>45.5850mm</t>
+          <t>33.0750mm</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1415,18 +1415,18 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>5.2189mm</t>
+          <t>2.7189mm</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1446,12 +1446,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>7.7189mm</t>
+          <t>5.2189mm</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1471,17 +1471,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10.2189mm</t>
+          <t>7.7189mm</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>45.5750mm</t>
+          <t>45.5850mm</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1496,17 +1496,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>12.7189mm</t>
+          <t>10.2189mm</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>45.5850mm</t>
+          <t>45.5750mm</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1521,17 +1521,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>45.2289mm</t>
+          <t>12.7189mm</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>9.0750mm</t>
+          <t>45.5850mm</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1540,23 +1540,23 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>13.2089mm</t>
+          <t>47.2089mm</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>15.0750mm</t>
+          <t>5.0750mm</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1565,23 +1565,23 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>27.7189mm</t>
+          <t>15.1390mm</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>19.0650mm</t>
+          <t>13.0828mm</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1590,23 +1590,23 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>45.2089mm</t>
+          <t>27.7189mm</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>12.0750mm</t>
+          <t>17.5850mm</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1615,23 +1615,23 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>45.2289mm</t>
+          <t>45.7089mm</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10.5750mm</t>
+          <t>11.0750mm</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1646,17 +1646,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>13.2089mm</t>
+          <t>46.2089mm</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>19.0750mm</t>
+          <t>8.0750mm</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1671,17 +1671,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>13.2089mm</t>
+          <t>15.1390mm</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>17.5750mm</t>
+          <t>20.5828mm</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1696,17 +1696,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>13.2089mm</t>
+          <t>15.1390mm</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>12.0750mm</t>
+          <t>17.0828mm</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1721,17 +1721,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>13.2089mm</t>
+          <t>28.7089mm</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>13.5750mm</t>
+          <t>2.5750mm</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1746,17 +1746,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SW1</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>24.2189mm</t>
+          <t>42.7089mm</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>47.5750mm</t>
+          <t>9.0750mm</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1765,23 +1765,23 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SW2</t>
+          <t>SW1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>28.7189mm</t>
+          <t>16.7189mm</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>47.5750mm</t>
+          <t>48.0750mm</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1796,17 +1796,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>SW2</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10.0989mm</t>
+          <t>20.7189mm</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>32.3250mm</t>
+          <t>48.0750mm</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1815,23 +1815,23 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>90</v>
+        <v>270</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>35.4689mm</t>
+          <t>10.0989mm</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>15.8250mm</t>
+          <t>32.3250mm</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1840,23 +1840,23 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>270</v>
+        <v>90</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>23.8489mm</t>
+          <t>35.4689mm</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>7.1250mm</t>
+          <t>15.8250mm</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1871,17 +1871,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>17.9189mm</t>
+          <t>22.3489mm</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>18.1250mm</t>
+          <t>7.6250mm</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1890,23 +1890,23 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0</v>
+        <v>270</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>38.9689mm</t>
+          <t>21.4189mm</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>36.1250mm</t>
+          <t>16.1250mm</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1915,31 +1915,56 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>U5</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>42.4689mm</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>36.1250mm</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>43.8439mm</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>19.8750mm</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>44.3439mm</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>22.8750mm</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>